<commit_message>
Fix payment and takhmeen update logic - use CASE instead of COALESCE
Issue: COALESCE doesn't update values to 0, causing old data to persist
Solution: Use CASE statements to properly handle null vs 0 values
- Payment update: Now correctly updates amt_rcv and amt_pending
- Takhmeen update: Now correctly updates takhmeen_amt and previous_amount_due
- Empty strings still don't overwrite existing data (intentional)
- Null values preserve existing data (intentional)

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015gjxBjc6nem1C85vnzkmCr
</commit_message>
<xml_diff>
--- a/fmb-data-updated-new.xlsx
+++ b/fmb-data-updated-new.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\saas-payment-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{51B7B7C3-3BE5-4C16-BDD7-340E7E1975AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C09E5ACC-D491-4D6E-8030-C4F53BB13143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C00B608F-BB65-4465-B56D-B4B91D48B788}"/>
+    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="10060" xr2:uid="{C00B608F-BB65-4465-B56D-B4B91D48B788}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="43">
   <si>
     <t xml:space="preserve">
 DAWOODI BOHRA JAMAAT TRUST - FATEMI MOHALLA POONA
@@ -83,13 +83,79 @@
     <t>DAROOS SUROOR SECTOR</t>
   </si>
   <si>
-    <t>A0027</t>
-  </si>
-  <si>
-    <t>ALIASGAR BHAI SHAIKH AKBERALI BHAI CHAIWALA</t>
-  </si>
-  <si>
-    <t>9x-25</t>
+    <t>A0043</t>
+  </si>
+  <si>
+    <t>MARYAM BAI MULLA ABBAS BHAI MERCHANT</t>
+  </si>
+  <si>
+    <t>Me-20</t>
+  </si>
+  <si>
+    <t>I0528</t>
+  </si>
+  <si>
+    <t>Mohammed bhai Abbas bhai Merchant</t>
+  </si>
+  <si>
+    <t>HUSAIN SECTOR</t>
+  </si>
+  <si>
+    <t>Sm-25</t>
+  </si>
+  <si>
+    <t>G0344</t>
+  </si>
+  <si>
+    <t>MULLA HUZEFA BHAI MOHAMMEDALI BHAI ANDAMANWALA</t>
+  </si>
+  <si>
+    <t>BABJI SECTOR</t>
+  </si>
+  <si>
+    <t>Me-28</t>
+  </si>
+  <si>
+    <t>G0374</t>
+  </si>
+  <si>
+    <t>SHAIKH ABBAS BHAI MULLA HEBATULLAH BHAI VASI</t>
+  </si>
+  <si>
+    <t>Sm-52</t>
+  </si>
+  <si>
+    <t>F0293</t>
+  </si>
+  <si>
+    <t>SHAIKH SAIFUDDIN BHAI MULLA IBRAHIM BHAI PATANWALA</t>
+  </si>
+  <si>
+    <t>HUTAIB SECTOR</t>
+  </si>
+  <si>
+    <t>Sm-69</t>
+  </si>
+  <si>
+    <t>NRI092</t>
+  </si>
+  <si>
+    <t>MOHAMMED BHAI MALWA</t>
+  </si>
+  <si>
+    <t>9x-16</t>
+  </si>
+  <si>
+    <t>I0442</t>
+  </si>
+  <si>
+    <t>SHAIKH AKBAR BHAI MULLA ABDULLAH BHAI PARDAWALA</t>
+  </si>
+  <si>
+    <t>NOOR SECTOR</t>
+  </si>
+  <si>
+    <t>Sm-97</t>
   </si>
 </sst>
 </file>
@@ -453,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43E2BDDB-3546-4361-8B4F-58F6AA70A255}">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.1796875" customWidth="1"/>
@@ -535,10 +601,10 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>50450029</v>
+        <v>30373990</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
@@ -555,25 +621,274 @@
       <c r="G3" t="s">
         <v>15</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" s="3">
+        <v>50000</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2">
+        <v>20000</v>
+      </c>
+      <c r="N3" s="2">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2">
+        <v>30320681</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="3">
+        <v>38750</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2">
+        <v>19250</v>
+      </c>
+      <c r="N4" s="2">
+        <v>19500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2">
+        <v>30377172</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="3">
+        <v>111000</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2">
+        <v>78000</v>
+      </c>
+      <c r="N5" s="2">
+        <v>33000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2">
+        <v>20359801</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="3">
+        <v>35000</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2">
+        <v>26000</v>
+      </c>
+      <c r="N6" s="2">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2">
+        <v>20303035</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="3">
+        <v>92000</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2">
+        <v>0</v>
+      </c>
+      <c r="M7" s="2">
+        <v>40000</v>
+      </c>
+      <c r="N7" s="2">
+        <v>52000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2">
+        <v>30373294</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="3">
-        <v>126792</v>
-      </c>
-      <c r="J3" s="2">
-        <v>0</v>
-      </c>
-      <c r="K3" s="3">
-        <v>0</v>
-      </c>
-      <c r="L3" s="2">
-        <v>0</v>
-      </c>
-      <c r="M3" s="2">
-        <v>126792</v>
-      </c>
-      <c r="N3" s="2">
+      <c r="I8" s="3">
+        <v>76000</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2">
+        <v>30000</v>
+      </c>
+      <c r="N8" s="2">
+        <v>46000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2">
+        <v>20325159</v>
+      </c>
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="3">
+        <v>72000</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2">
+        <v>72000</v>
+      </c>
+      <c r="N9" s="2">
         <v>0</v>
       </c>
     </row>

</xml_diff>